<commit_message>
Ajuste no print do mapa e alterações nos dados da tabela enemy
</commit_message>
<xml_diff>
--- a/dist/OWPick/_internal/heroes enemy.xlsx
+++ b/dist/OWPick/_internal/heroes enemy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DAVI\Projeto\Overwatch\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F8BBFA4-FFDD-4C04-9599-27ED49C93351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA2E37CE-B071-486A-B8A9-FD7F65BFD683}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1077,7 +1077,7 @@
         <v>0</v>
       </c>
       <c r="AF4" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG4" s="3">
         <v>0</v>
@@ -1110,7 +1110,7 @@
         <v>0</v>
       </c>
       <c r="AQ4" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AR4" s="3">
         <v>0</v>
@@ -1697,7 +1697,7 @@
         <v>0</v>
       </c>
       <c r="AF8" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG8" s="3">
         <v>0</v>
@@ -1733,7 +1733,7 @@
         <v>0</v>
       </c>
       <c r="AR8" s="3">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="AS8" s="3">
         <v>1</v>

</xml_diff>

<commit_message>
Alterações nas planilha e nova funcionalidade que remove a pontuação dos mapas na soma final
</commit_message>
<xml_diff>
--- a/dist/OWPick/_internal/heroes enemy.xlsx
+++ b/dist/OWPick/_internal/heroes enemy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DAVI\Projeto\Overwatch\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA2E37CE-B071-486A-B8A9-FD7F65BFD683}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D255E467-2780-420A-992E-AA0F87433D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1172,7 +1172,7 @@
         <v>-1</v>
       </c>
       <c r="L5" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M5" s="3">
         <v>0</v>

</xml_diff>

<commit_message>
v1.0.6 - Updates na planilha enemies e allys
Updates na planilha enemies e allys
</commit_message>
<xml_diff>
--- a/dist/OWPick/_internal/heroes enemy.xlsx
+++ b/dist/OWPick/_internal/heroes enemy.xlsx
@@ -789,7 +789,7 @@
         <v>0</v>
       </c>
       <c r="D3" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" s="2">
         <v>0</v>
@@ -801,7 +801,7 @@
         <v>1</v>
       </c>
       <c r="H3" s="2">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="I3" s="2">
         <v>2</v>
@@ -825,7 +825,7 @@
         <v>1</v>
       </c>
       <c r="P3" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q3" s="2">
         <v>-2</v>
@@ -944,7 +944,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D4" s="2">
         <v>0</v>
@@ -1001,7 +1001,7 @@
         <v>1</v>
       </c>
       <c r="V4" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W4" s="2">
         <v>0</v>
@@ -1040,7 +1040,7 @@
         <v>0</v>
       </c>
       <c r="AI4" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ4" s="2">
         <v>0</v>
@@ -1299,7 +1299,7 @@
         <v>-2</v>
       </c>
       <c r="P6" s="2">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="Q6" s="2">
         <v>-1</v>
@@ -1457,7 +1457,7 @@
         <v>0</v>
       </c>
       <c r="P7" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="Q7" s="2">
         <v>0</v>
@@ -1490,7 +1490,7 @@
         <v>1</v>
       </c>
       <c r="AA7" s="2">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AB7" s="2">
         <v>-1</v>
@@ -1576,7 +1576,7 @@
         <v>-1</v>
       </c>
       <c r="C8" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" s="2">
         <v>-1</v>
@@ -1618,7 +1618,7 @@
         <v>-1</v>
       </c>
       <c r="Q8" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R8" s="2">
         <v>0</v>
@@ -1773,7 +1773,7 @@
         <v>0</v>
       </c>
       <c r="P9" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="2">
         <v>0</v>
@@ -1931,7 +1931,7 @@
         <v>1</v>
       </c>
       <c r="P10" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q10" s="2">
         <v>1</v>
@@ -2089,7 +2089,7 @@
         <v>0</v>
       </c>
       <c r="P11" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q11" s="2">
         <v>1</v>
@@ -2447,7 +2447,7 @@
         <v>1</v>
       </c>
       <c r="AD13" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE13" s="2">
         <v>1</v>
@@ -2513,7 +2513,7 @@
         <v>-1</v>
       </c>
       <c r="AZ13" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
@@ -2829,7 +2829,7 @@
         <v>-2</v>
       </c>
       <c r="AZ15" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
@@ -2846,7 +2846,7 @@
         <v>0</v>
       </c>
       <c r="E16" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" s="2">
         <v>2</v>
@@ -2885,10 +2885,10 @@
         <v>-2</v>
       </c>
       <c r="R16" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S16" s="2">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="T16" s="2">
         <v>0</v>
@@ -2918,7 +2918,7 @@
         <v>0</v>
       </c>
       <c r="AC16" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD16" s="2">
         <v>0</v>
@@ -2942,7 +2942,7 @@
         <v>1</v>
       </c>
       <c r="AK16" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AL16" s="2">
         <v>0</v>
@@ -2966,7 +2966,7 @@
         <v>-2</v>
       </c>
       <c r="AS16" s="2">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AT16" s="2">
         <v>-2</v>
@@ -2975,13 +2975,13 @@
         <v>0</v>
       </c>
       <c r="AV16" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AW16" s="2">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="AX16" s="2">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AY16" s="2">
         <v>0</v>
@@ -3013,7 +3013,7 @@
         <v>0</v>
       </c>
       <c r="H17" s="2">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I17" s="2">
         <v>-1</v>
@@ -3037,7 +3037,7 @@
         <v>0</v>
       </c>
       <c r="P17" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q17" s="2">
         <v>0</v>
@@ -3139,7 +3139,7 @@
         <v>-1</v>
       </c>
       <c r="AX17" s="2">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AY17" s="2">
         <v>0</v>
@@ -3159,7 +3159,7 @@
         <v>0</v>
       </c>
       <c r="D18" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18" s="2">
         <v>1</v>
@@ -3353,7 +3353,7 @@
         <v>1</v>
       </c>
       <c r="P19" s="2">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="Q19" s="2">
         <v>1</v>
@@ -3511,7 +3511,7 @@
         <v>0</v>
       </c>
       <c r="P20" s="2">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="Q20" s="2">
         <v>-1</v>
@@ -3747,7 +3747,7 @@
         <v>-1</v>
       </c>
       <c r="AP21" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AQ21" s="2">
         <v>-1</v>
@@ -3791,7 +3791,7 @@
         <v>-1</v>
       </c>
       <c r="D22" s="2">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="E22" s="2">
         <v>0</v>
@@ -3827,7 +3827,7 @@
         <v>0</v>
       </c>
       <c r="P22" s="2">
-        <v>-2</v>
+        <v>2</v>
       </c>
       <c r="Q22" s="2">
         <v>-2</v>
@@ -3949,7 +3949,7 @@
         <v>0</v>
       </c>
       <c r="D23" s="2">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="E23" s="2">
         <v>0</v>
@@ -4143,7 +4143,7 @@
         <v>0</v>
       </c>
       <c r="P24" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="Q24" s="2">
         <v>0</v>
@@ -4301,7 +4301,7 @@
         <v>1</v>
       </c>
       <c r="P25" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q25" s="2">
         <v>-1</v>
@@ -4590,7 +4590,7 @@
         <v>-1</v>
       </c>
       <c r="G27" s="2">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="H27" s="2">
         <v>0</v>
@@ -4671,7 +4671,7 @@
         <v>2</v>
       </c>
       <c r="AH27" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI27" s="2">
         <v>0</v>
@@ -5091,7 +5091,7 @@
         <v>1</v>
       </c>
       <c r="P30" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q30" s="2">
         <v>-2</v>
@@ -5371,7 +5371,7 @@
         <v>0</v>
       </c>
       <c r="D32" s="2">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="E32" s="2">
         <v>0</v>
@@ -5407,7 +5407,7 @@
         <v>1</v>
       </c>
       <c r="P32" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q32" s="2">
         <v>0</v>
@@ -5565,7 +5565,7 @@
         <v>0</v>
       </c>
       <c r="P33" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="Q33" s="2">
         <v>-2</v>
@@ -5723,7 +5723,7 @@
         <v>0</v>
       </c>
       <c r="P34" s="2">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="Q34" s="2">
         <v>-2</v>
@@ -5756,7 +5756,7 @@
         <v>0</v>
       </c>
       <c r="AA34" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AB34" s="2">
         <v>0</v>
@@ -5845,7 +5845,7 @@
         <v>0</v>
       </c>
       <c r="D35" s="2">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="E35" s="2">
         <v>0</v>
@@ -6197,7 +6197,7 @@
         <v>0</v>
       </c>
       <c r="P37" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q37" s="2">
         <v>0</v>
@@ -6561,7 +6561,7 @@
         <v>2</v>
       </c>
       <c r="AF39" s="2">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AG39" s="2">
         <v>1</v>
@@ -6671,7 +6671,7 @@
         <v>-1</v>
       </c>
       <c r="P40" s="2">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="Q40" s="2">
         <v>0</v>
@@ -6931,7 +6931,7 @@
         <v>2</v>
       </c>
       <c r="AX41" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AY41" s="2">
         <v>-1</v>
@@ -7002,7 +7002,7 @@
         <v>1</v>
       </c>
       <c r="U42" s="2">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="V42" s="2">
         <v>0</v>
@@ -7408,7 +7408,7 @@
         <v>-1</v>
       </c>
       <c r="AY44" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AZ44" s="2">
         <v>2</v>
@@ -7619,7 +7619,7 @@
         <v>0</v>
       </c>
       <c r="P46" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q46" s="2">
         <v>0</v>
@@ -7777,7 +7777,7 @@
         <v>-1</v>
       </c>
       <c r="P47" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q47" s="2">
         <v>0</v>
@@ -8254,7 +8254,7 @@
         <v>0</v>
       </c>
       <c r="Q50" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R50" s="2">
         <v>-2</v>
@@ -8326,7 +8326,7 @@
         <v>-2</v>
       </c>
       <c r="AO50" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP50" s="2">
         <v>0</v>
@@ -8493,7 +8493,7 @@
         <v>-1</v>
       </c>
       <c r="AR51" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AS51" s="2">
         <v>1</v>
@@ -8525,16 +8525,16 @@
         <v>51</v>
       </c>
       <c r="B52" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C52" s="2">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="D52" s="2">
         <v>0</v>
       </c>
       <c r="E52" s="2">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="F52" s="2">
         <v>1</v>
@@ -8543,13 +8543,13 @@
         <v>2</v>
       </c>
       <c r="H52" s="2">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="I52" s="2">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="J52" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K52" s="2">
         <v>1</v>
@@ -8558,16 +8558,16 @@
         <v>-1</v>
       </c>
       <c r="M52" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="N52" s="2">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="O52" s="2">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="P52" s="2">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="Q52" s="2">
         <v>-2</v>
@@ -8678,7 +8678,11 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="53" ht="15.75" customHeight="1"/>
+    <row r="53" ht="15.75" customHeight="1">
+      <c r="J53" s="2">
+        <v>-1</v>
+      </c>
+    </row>
     <row r="54" ht="15.75" customHeight="1"/>
     <row r="55" ht="15.75" customHeight="1"/>
     <row r="56" ht="15.75" customHeight="1"/>
@@ -9628,8 +9632,13 @@
     <row r="1000" ht="15.75" customHeight="1"/>
     <row r="1001" ht="15.75" customHeight="1"/>
   </sheetData>
+  <conditionalFormatting sqref="J53">
+    <cfRule priority="1" dxfId="0" type="expression">
+      <formula>J53&lt;&gt;-INDIRECT(ADDRESS(MATCH(J$1,$A:$A,0),MATCH($A53,$1:$1,0)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B2:AZ52">
-    <cfRule priority="1" dxfId="0" type="expression">
+    <cfRule priority="2" dxfId="0" type="expression">
       <formula>B2&lt;&gt;-INDIRECT(ADDRESS(MATCH(B$1,$A:$A,0),MATCH($A2,$1:$1,0)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>